<commit_message>
Add submission attempts and update exam workflows
Normalize submission files and track attempts, expose only the latest submission, and release grading results after exams close. Update roster imports to enroll existing students only, add demo account seeding, and improve exam Markdown previews and student-facing pages.
</commit_message>
<xml_diff>
--- a/demo/examples/studentImport/sinh_vien_test_AITA-TEST-001.xlsx
+++ b/demo/examples/studentImport/sinh_vien_test_AITA-TEST-001.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9615329F-5778-4E7D-B4BD-286136901485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="3072" yWindow="3072" windowWidth="17280" windowHeight="9912" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sinh viên" state="visible" r:id="rId4"/>
+    <sheet name="Sinh viên" sheetId="2" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sinh viên'!$A1:$B11</definedName>
-  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Email</t>
   </si>
@@ -56,72 +57,33 @@
   </si>
   <si>
     <t>Vũ Thị Thu Trang</t>
-  </si>
-  <si>
-    <t>student.test07@fpt.edu.vn</t>
-  </si>
-  <si>
-    <t>Đặng Quốc Bảo</t>
-  </si>
-  <si>
-    <t>student.test08@fpt.edu.vn</t>
-  </si>
-  <si>
-    <t>Bùi Khánh Linh</t>
-  </si>
-  <si>
-    <t>student.test09@fpt.edu.vn</t>
-  </si>
-  <si>
-    <t>Đỗ Hải Đăng</t>
-  </si>
-  <si>
-    <t>student.test10@fpt.edu.vn</t>
-  </si>
-  <si>
-    <t>Ngô Phương Thảo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF1F2937"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1D4ED8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -136,17 +98,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,18 +439,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85C942D0-63B0-482B-8147-E6B2F963D3DE}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -504,88 +455,55 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
-  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>